<commit_message>
scan: seg2 2026-07-10 20:13 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq3_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq3_2026-07-09.xlsx
@@ -7364,21 +7364,21 @@
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
-        <v>3018</v>
+        <v>3045</v>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>隆銘綠能</t>
+          <t>台灣大</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v/>
       </c>
       <c r="D131" s="2" t="n">
-        <v>509.2031715851631</v>
+        <v>509.5105669229774</v>
       </c>
       <c r="E131" s="2" t="n">
-        <v>12.05</v>
+        <v>108.5</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -7389,16 +7389,16 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>52.96042354178515</v>
+        <v>28.61825215344104</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>14.00411353344998</v>
+        <v>24.1905696067152</v>
       </c>
       <c r="J131" s="2" t="n">
-        <v>1.782279900691022</v>
+        <v>3.35105669229774</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L131" s="2" t="n">
         <v>0</v>
@@ -7407,31 +7407,31 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>0.129868093056733</v>
+        <v>-1.125708078864336</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
-        <v>2546</v>
+        <v>3018</v>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>根基</t>
+          <t>隆銘綠能</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>505.6918777352019</v>
+        <v>509.2031715851631</v>
       </c>
       <c r="E132" s="2" t="n">
-        <v>92.2</v>
+        <v>12.05</v>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
@@ -7442,16 +7442,16 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>49.9323048554422</v>
+        <v>52.96042354178515</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>32.60395640960779</v>
+        <v>14.00411353344998</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>0.4950859361523834</v>
+        <v>1.782279900691022</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L132" s="2" t="n">
         <v>0</v>
@@ -7460,31 +7460,31 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.469436052221289</v>
+        <v>0.129868093056733</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>2471</v>
+        <v>2546</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>資通</t>
+          <t>根基</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>503.012503951619</v>
+        <v>505.6918777352019</v>
       </c>
       <c r="E133" s="2" t="n">
-        <v>53.2</v>
+        <v>92.2</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -7495,16 +7495,16 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>51.51269854591602</v>
+        <v>49.9323048554422</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>11.9493841565906</v>
+        <v>32.60395640960779</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>0.4179962674339422</v>
+        <v>0.4950859361523834</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L133" s="2" t="n">
         <v>0</v>
@@ -7513,31 +7513,31 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-0.0016340680262111</v>
+        <v>-0.469436052221289</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>2459</v>
+        <v>2471</v>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>敦吉</t>
+          <t>資通</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v/>
       </c>
       <c r="D134" s="2" t="n">
-        <v>501.0279350152362</v>
+        <v>503.012503951619</v>
       </c>
       <c r="E134" s="2" t="n">
-        <v>63.7</v>
+        <v>53.2</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -7548,13 +7548,13 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>39.33170025812593</v>
+        <v>51.51269854591602</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>24.2600086006961</v>
+        <v>11.9493841565906</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>0.2725027174650308</v>
+        <v>0.4179962674339422</v>
       </c>
       <c r="K134" s="2" t="n">
         <v>0</v>
@@ -7566,31 +7566,31 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>-0.0429512561549253</v>
+        <v>-0.0016340680262111</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>3073</v>
+        <v>2459</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>天方能源</t>
+          <t>敦吉</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v/>
       </c>
       <c r="D135" s="2" t="n">
-        <v>499.2337368577561</v>
+        <v>501.0279350152362</v>
       </c>
       <c r="E135" s="2" t="n">
-        <v>22</v>
+        <v>63.7</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -7601,13 +7601,13 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>50.7709844566271</v>
+        <v>39.33170025812593</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>20.47660706899832</v>
+        <v>24.2600086006961</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>0.6276859944218266</v>
+        <v>0.2725027174650308</v>
       </c>
       <c r="K135" s="2" t="n">
         <v>0</v>
@@ -7619,31 +7619,31 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>0.0916149920180276</v>
+        <v>-0.0429512561549253</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>3041</v>
+        <v>3073</v>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>揚智</t>
+          <t>天方能源</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v/>
       </c>
       <c r="D136" s="2" t="n">
-        <v>498.4394930957397</v>
+        <v>499.2337368577561</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>26.45</v>
+        <v>22</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -7654,13 +7654,13 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>46.79258800013102</v>
+        <v>50.7709844566271</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>21.62521832728444</v>
+        <v>20.47660706899832</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0.272872747042126</v>
+        <v>0.6276859944218266</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>0</v>
@@ -7672,31 +7672,31 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>-0.3574170756442113</v>
+        <v>0.0916149920180276</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>3002</v>
+        <v>3041</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>歐格</t>
+          <t>揚智</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>497.2449589827172</v>
+        <v>498.4394930957397</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>20.45</v>
+        <v>26.45</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -7707,13 +7707,13 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>48.96783905627235</v>
+        <v>46.79258800013102</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>35.60455543350986</v>
+        <v>21.62521832728444</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>0.2916001953823394</v>
+        <v>0.272872747042126</v>
       </c>
       <c r="K137" s="2" t="n">
         <v>0</v>
@@ -7725,31 +7725,31 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>-0.1917893926327997</v>
+        <v>-0.3574170756442113</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>2731</v>
+        <v>3002</v>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>雄獅</t>
+          <t>歐格</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v/>
       </c>
       <c r="D138" s="2" t="n">
-        <v>496.6071263236449</v>
+        <v>497.2449589827172</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>145.5</v>
+        <v>20.45</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -7760,13 +7760,13 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>30.88348934736115</v>
+        <v>48.96783905627235</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>23.33322271680851</v>
+        <v>35.60455543350986</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>0.9235818372441584</v>
+        <v>0.2916001953823394</v>
       </c>
       <c r="K138" s="2" t="n">
         <v>0</v>
@@ -7778,31 +7778,31 @@
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>-0.0951940029337965</v>
+        <v>-0.1917893926327997</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>2608</v>
+        <v>2731</v>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>嘉里大榮</t>
+          <t>雄獅</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>495.8506033487794</v>
+        <v>496.6071263236449</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>29.45</v>
+        <v>145.5</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -7813,16 +7813,16 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>54.13420944703902</v>
+        <v>30.88348934736115</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>19.4644188259638</v>
+        <v>23.33322271680851</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>0.5327558711538301</v>
+        <v>0.9235818372441584</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L139" s="2" t="n">
         <v>0</v>
@@ -7831,31 +7831,31 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>0.0715435705266575</v>
+        <v>-0.0951940029337965</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>2462</v>
+        <v>2608</v>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>良得電</t>
+          <t>嘉里大榮</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v/>
       </c>
       <c r="D140" s="2" t="n">
-        <v>490.0669938718079</v>
+        <v>495.8506033487794</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>22.85</v>
+        <v>29.45</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -7866,16 +7866,16 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>42.00613390511628</v>
+        <v>54.13420944703902</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>17.98530594241905</v>
+        <v>19.4644188259638</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>0.3790319613823146</v>
+        <v>0.5327558711538301</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L140" s="2" t="n">
         <v>0</v>
@@ -7884,31 +7884,31 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>-0.3037596928425445</v>
+        <v>0.0715435705266575</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
-        <v>3045</v>
+        <v>2462</v>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>台灣大</t>
+          <t>良得電</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v/>
       </c>
       <c r="D141" s="2" t="n">
-        <v>489.5105669229774</v>
+        <v>490.0669938718079</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>108.5</v>
+        <v>22.85</v>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
@@ -7919,16 +7919,16 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>28.61825215344104</v>
+        <v>42.00613390511628</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>24.1905696067152</v>
+        <v>17.98530594241905</v>
       </c>
       <c r="J141" s="2" t="n">
-        <v>3.35105669229774</v>
+        <v>0.3790319613823146</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L141" s="2" t="n">
         <v>0</v>
@@ -7937,11 +7937,11 @@
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>-1.125708078864336</v>
+        <v>-0.3037596928425445</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>

</xml_diff>